<commit_message>
Initial commit - Dev Guardian AI security scanner
</commit_message>
<xml_diff>
--- a/docs/Sea_GenAI_Sec_Spv_Agent_LC.xlsx
+++ b/docs/Sea_GenAI_Sec_Spv_Agent_LC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sea_GenAI_Sec_Spv_Agent_LC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev_Guardian\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B748E23B-AD77-4921-A6AC-846EB979FAD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDDEBB1-95DF-402D-AB9E-B14F775103C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{889FE935-10F9-40CD-A804-48CF79D50F19}"/>
+    <workbookView xWindow="42870" yWindow="0" windowWidth="14805" windowHeight="15510" xr2:uid="{889FE935-10F9-40CD-A804-48CF79D50F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>